<commit_message>
feat: ödeme importuna Durum kolonu ekle (Tamamlandı/Beklemede)
- Excel'de yeni kolon: "Durum" — Tamamlandı veya Beklemede
- Boş bırakılırsa varsayılan Tamamlandı
- Önizleme tablosunda statü badge'i gösteriliyor
- Excel şablon güncellendi

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/templates/odeme-import-sablonu.xlsx
+++ b/public/templates/odeme-import-sablonu.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:G3"/>
   <cols>
     <col min="1" max="1" width="15.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
@@ -406,6 +406,7 @@
     <col min="4" max="4" width="40.83203125" customWidth="1"/>
     <col min="5" max="5" width="30.83203125" customWidth="1"/>
     <col min="6" max="6" width="15.83203125" customWidth="1"/>
+    <col min="7" max="7" width="15.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -427,6 +428,9 @@
       <c r="F1" t="str">
         <v>Ödeme Tarihi</v>
       </c>
+      <c r="G1" t="str">
+        <v>Durum</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -447,6 +451,9 @@
       <c r="F2" t="str">
         <v>22.01.2026</v>
       </c>
+      <c r="G2" t="str">
+        <v>Tamamlandı</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -467,10 +474,13 @@
       <c r="F3" t="str">
         <v/>
       </c>
+      <c r="G3" t="str">
+        <v>Beklemede</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G3"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -481,7 +491,7 @@
   <cols>
     <col min="1" max="1" width="20.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
-    <col min="3" max="3" width="40.83203125" customWidth="1"/>
+    <col min="3" max="3" width="50.83203125" customWidth="1"/>
     <col min="4" max="4" width="30.83203125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -605,32 +615,41 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v/>
+        <v>Durum</v>
+      </c>
+      <c r="B12" t="str">
+        <v>HAYIR</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Tamamlandı veya Beklemede (varsayılan: Tamamlandı)</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Tamamlandı</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>ÖNEMLİ NOTLAR:</v>
+        <v/>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>1. Alıcı adı sistemdeki kullanıcı veya personel kaydıyla birebir eşleşmelidir.</v>
+        <v>ÖNEMLİ NOTLAR:</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>2. Kişinin ilgili projede yeterli bakiyesi olmalıdır.</v>
+        <v>1. Alıcı adı sistemdeki kullanıcı veya personel kaydıyla eşleşmelidir (fuzzy matching desteklenir).</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>3. Aynı kişi birden fazla satırda yer alabilir; bakiye kümülatif kontrol edilir.</v>
+        <v>2. Durum boş bırakılırsa Tamamlandı olarak işlenir.</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>4. Ödeme talimatı "pending" statüsünde oluşturulur, bakiye reserve edilir.</v>
+        <v>3. Aynı kişi birden fazla satırda yer alabilir.</v>
       </c>
     </row>
   </sheetData>

</xml_diff>